<commit_message>
Keep only test analyst deliverables required by sprint 2 assignment
</commit_message>
<xml_diff>
--- a/docs/sprint2/requirements-defects.xlsx
+++ b/docs/sprint2/requirements-defects.xlsx
@@ -2,10 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реєстр" sheetId="1" r:id="R3f137d034f8b44e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Розподіл розділів" sheetId="2" r:id="R5d5c15d6fbe74f73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Спірні" sheetId="3" r:id="Rd013b84dafb34a39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Підсумок" sheetId="4" r:id="R498c5d59b5a640fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реєстр" sheetId="1" r:id="Rc902b576e9ff4dd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Розподіл розділів" sheetId="2" r:id="R6e15ff85fb064ee6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Спірні" sheetId="3" r:id="Rc54dfbde20f848b6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,7 +18,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="4">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -41,14 +40,8 @@
       <x:color rgb="FF305496"/>
       <x:name val="Arial"/>
     </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="10"/>
-      <x:color rgb="FF223044"/>
-      <x:name val="Arial"/>
-    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="3">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -58,11 +51,6 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF305496"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE9EFF7"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -78,7 +66,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="30">
+  <x:cellXfs count="23">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -138,32 +126,11 @@
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="4">
+  <x:dxfs count="3">
     <x:dxf>
       <x:fill>
         <x:patternFill patternType="solid">
@@ -182,17 +149,6 @@
       <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFFF2CC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF9C0006"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -1269,7 +1225,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c94d2b8248a40bd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae4d02902d024c44"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1928,223 +1884,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80d64b3b63ce4c8c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0153f4c7cc774f06"/>
   </x:tableParts>
 </x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="29" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="8" t="str">
-        <x:v>Критерій</x:v>
-      </x:c>
-      <x:c r="B1" s="8" t="str">
-        <x:v>Прийнято</x:v>
-      </x:c>
-      <x:c r="C1" s="8" t="str">
-        <x:v>Відхилено у «Спірні»</x:v>
-      </x:c>
-      <x:c r="D1" s="8" t="str">
-        <x:v>Мінімум</x:v>
-      </x:c>
-      <x:c r="E1" s="8" t="str">
-        <x:v>Норматив кількості</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="4" t="str">
-        <x:v>Однозначність</x:v>
-      </x:c>
-      <x:c r="B2" s="10" t="n">
-        <x:f>COUNTIFS('Реєстр'!$C$2:$C$28,A2,'Реєстр'!$G$2:$G$28,"прийнято")</x:f>
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C2" s="10" t="n">
-        <x:f>COUNTIFS('Спірні'!$C$2:$C$5,A2,'Спірні'!$H$2:$H$5,"відхилено після обговорення")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D2" s="10" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E2" s="23" t="str">
-        <x:f>IF(B2&gt;=D2,"Виконано","Недостатньо")</x:f>
-        <x:v>Виконано</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="34" customHeight="1">
-      <x:c r="A3" s="4" t="str">
-        <x:v>Повнота</x:v>
-      </x:c>
-      <x:c r="B3" s="10" t="n">
-        <x:f>COUNTIFS('Реєстр'!$C$2:$C$28,A3,'Реєстр'!$G$2:$G$28,"прийнято")</x:f>
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C3" s="10" t="n">
-        <x:f>COUNTIFS('Спірні'!$C$2:$C$5,A3,'Спірні'!$H$2:$H$5,"відхилено після обговорення")</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D3" s="10" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E3" s="23" t="str">
-        <x:f>IF(B3&gt;=D3,"Виконано","Недостатньо")</x:f>
-        <x:v>Виконано</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="34" customHeight="1">
-      <x:c r="A4" s="4" t="str">
-        <x:v>Несуперечливість</x:v>
-      </x:c>
-      <x:c r="B4" s="10" t="n">
-        <x:f>COUNTIFS('Реєстр'!$C$2:$C$28,A4,'Реєстр'!$G$2:$G$28,"прийнято")</x:f>
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C4" s="10" t="n">
-        <x:f>COUNTIFS('Спірні'!$C$2:$C$5,A4,'Спірні'!$H$2:$H$5,"відхилено після обговорення")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D4" s="10" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E4" s="23" t="str">
-        <x:f>IF(B4&gt;=D4,"Виконано","Недостатньо")</x:f>
-        <x:v>Виконано</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="4" t="str">
-        <x:v>Простежуваність</x:v>
-      </x:c>
-      <x:c r="B5" s="10" t="n">
-        <x:f>COUNTIFS('Реєстр'!$C$2:$C$28,A5,'Реєстр'!$G$2:$G$28,"прийнято")</x:f>
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C5" s="10" t="n">
-        <x:f>COUNTIFS('Спірні'!$C$2:$C$5,A5,'Спірні'!$H$2:$H$5,"відхилено після обговорення")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D5" s="10" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E5" s="23" t="str">
-        <x:f>IF(B5&gt;=D5,"Виконано","Недостатньо")</x:f>
-        <x:v>Виконано</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="34" customHeight="1">
-      <x:c r="A6" s="4" t="str">
-        <x:v>Здійсненність</x:v>
-      </x:c>
-      <x:c r="B6" s="10" t="n">
-        <x:f>COUNTIFS('Реєстр'!$C$2:$C$28,A6,'Реєстр'!$G$2:$G$28,"прийнято")</x:f>
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C6" s="10" t="n">
-        <x:f>COUNTIFS('Спірні'!$C$2:$C$5,A6,'Спірні'!$H$2:$H$5,"відхилено після обговорення")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D6" s="10" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E6" s="23" t="str">
-        <x:f>IF(B6&gt;=D6,"Виконано","Недостатньо")</x:f>
-        <x:v>Виконано</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="34" customHeight="1">
-      <x:c r="A7" s="4" t="str">
-        <x:v>Тестопридатність</x:v>
-      </x:c>
-      <x:c r="B7" s="10" t="n">
-        <x:f>COUNTIFS('Реєстр'!$C$2:$C$28,A7,'Реєстр'!$G$2:$G$28,"прийнято")</x:f>
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C7" s="10" t="n">
-        <x:f>COUNTIFS('Спірні'!$C$2:$C$5,A7,'Спірні'!$H$2:$H$5,"відхилено після обговорення")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D7" s="10" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E7" s="23" t="str">
-        <x:f>IF(B7&gt;=D7,"Виконано","Недостатньо")</x:f>
-        <x:v>Виконано</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="34" customHeight="1">
-      <x:c r="A8" s="27" t="str">
-        <x:v>Усього</x:v>
-      </x:c>
-      <x:c r="B8" s="28" t="n">
-        <x:f>SUM(B2:B7)</x:f>
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="C8" s="28" t="n">
-        <x:f>SUM(C2:C7)</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D8" s="28" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E8" s="29" t="str">
-        <x:f>IF(B8&gt;=D8,"Виконано","Недостатньо")</x:f>
-        <x:v>Виконано</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="30" customHeight="1">
-      <x:c r="A10" s="21" t="str">
-        <x:v>Примітка</x:v>
-      </x:c>
-      <x:c r="B10" s="21" t="str">
-        <x:v>Пояснення</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="68" customHeight="1">
-      <x:c r="A11" s="3" t="str">
-        <x:v>Прийняті дефекти</x:v>
-      </x:c>
-      <x:c r="B11" s="3" t="str">
-        <x:v>27 записів у реєстрі; відхилений №28 збережено лише на аркуші «Спірні» і не зараховано до нормативу.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="68" customHeight="1">
-      <x:c r="A12" s="3" t="str">
-        <x:v>Класифікація №27</x:v>
-      </x:c>
-      <x:c r="B12" s="3" t="str">
-        <x:v>Редакторськи змінено з повноти на несуперечливість за §4.1: виправлення прибирає суперечливу обіцянку. Вихідне рішення збережено у «Спірні».</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="68" customHeight="1">
-      <x:c r="A13" s="3" t="str">
-        <x:v>Погодження</x:v>
-      </x:c>
-      <x:c r="B13" s="3" t="str">
-        <x:v>Позначка «прийнято» стосується дефекту за спільним реєстром. Непідтверджені формулювання позначені в реєстрі й SRS; питання наведено у «Спірні».</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="68" customHeight="1">
-      <x:c r="A14" s="3" t="str">
-        <x:v>Дата редакції</x:v>
-      </x:c>
-      <x:c r="B14" s="3" t="str">
-        <x:v>10.10.2026</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:conditionalFormatting sqref="E2:E8">
-    <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Недостатньо"/>
-  </x:conditionalFormatting>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Address requirements registry review for defects 27 and 11/26
</commit_message>
<xml_diff>
--- a/docs/sprint2/requirements-defects.xlsx
+++ b/docs/sprint2/requirements-defects.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реєстр" sheetId="1" r:id="Rc902b576e9ff4dd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Розподіл розділів" sheetId="2" r:id="R6e15ff85fb064ee6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Спірні" sheetId="3" r:id="Rc54dfbde20f848b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реєстр" sheetId="1" r:id="R0067e98c26e94903"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Розподіл розділів" sheetId="2" r:id="Rca94b90da58843f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Спірні" sheetId="3" r:id="R7eda1c119a9a4258"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -133,21 +133,21 @@
   <x:dxfs count="3">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -180,14 +180,14 @@
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Кандидат"/>
     <x:tableColumn id="2" name="ID / місце"/>
-    <x:tableColumn id="3" name="Критерій у джерелі"/>
-    <x:tableColumn id="4" name="Опис і пункт чек-листа із джерела"/>
+    <x:tableColumn id="3" name="Критерій у поточній редакції"/>
+    <x:tableColumn id="4" name="Опис і пункт чек-листа"/>
     <x:tableColumn id="5" name="Пропозиція із джерела"/>
     <x:tableColumn id="6" name="Аргументи із джерела"/>
     <x:tableColumn id="7" name="Хто знайшов"/>
     <x:tableColumn id="8" name="Статус рішення"/>
     <x:tableColumn id="9" name="№ дефекту"/>
-    <x:tableColumn id="10" name="Рішення у джерелі / редакторська примітка"/>
+    <x:tableColumn id="10" name="Поточна примітка / історія рішення"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -735,7 +735,7 @@
         <x:v>F-110: доставка 120 грн, «для замовлень від 2000 грн доставка безкоштовна»; BL-60: безкоштовна, якщо «сума після знижки не менша за 1500 грн». Різні поріг і база розрахунку. Підстава: Несуперечливість (п. 2); §4.4.</x:v>
       </x:c>
       <x:c r="E12" s="4" t="str">
-        <x:v>Оформлення замовлення складається з чотирьох кроків: «Cart» → «Sign in» → «Billing Address» → «Payment». Неавторизований покупець на кроці 2 входить або реєструється; на кроці 3 підтверджує адресу доставки (вулиця, місто, область, країна, поштовий індекс); на кроці 4 обирає спосіб оплати (банківський переказ, оплата при отриманні, кредитна картка, «купити зараз — заплатити пізніше», подарункова картка) і підтверджує замовлення. Підсумок замовлення містить суму товарів і вартість доставки. Вартість доставки визначається за BL-60: 120,00 грн; 0,00 грн, якщо сума після знижки не менша за 1500,00 грн. Рядки знижки за обсягом і за промокодом з’являються після інтеграції модуля (розділ 5) в інтерфейс. Застосування правила BL-60 до поточного інтерфейсу до інтеграції модуля та порядок урахування знижок потребують підтвердження замовником. Після підтвердження замовлення система показує повідомлення з номером рахунку-інвойсу.</x:v>
+        <x:v>Вартість доставки визначається за BL-60: 120,00 грн; 0,00 грн, якщо сума після знижки не менша за 1500,00 грн. Застосування правила BL-60 до поточного інтерфейсу до інтеграції модуля потребує підтвердження замовником.</x:v>
       </x:c>
       <x:c r="F12" s="4" t="str">
         <x:v>Бобров Павло (КТ)</x:v>
@@ -747,7 +747,7 @@
         <x:v>3. Функціональні</x:v>
       </x:c>
       <x:c r="I12" s="4" t="str">
-        <x:v>Потребує підтвердження замовником: Застосування BL-60 до поточного інтерфейсу і порядок урахування знижок.</x:v>
+        <x:v>Потребує підтвердження замовником: застосування BL-60 до поточного інтерфейсу до інтеграції модуля.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="80" customHeight="1">
@@ -1170,7 +1170,7 @@
         <x:v>Розд. 2.3: модуль програми лояльності «в поточній версії ще не інтегрований в інтерфейс»; F-110: підсумок замовлення «містить … знижку за обсягом, знижку за промокодом» — у поточній версії цих рядків бути не може. Підстава: Несуперечливість (п. 2); §4.4.</x:v>
       </x:c>
       <x:c r="E27" s="4" t="str">
-        <x:v>Оформлення замовлення складається з чотирьох кроків: «Cart» → «Sign in» → «Billing Address» → «Payment». Неавторизований покупець на кроці 2 входить або реєструється; на кроці 3 підтверджує адресу доставки (вулиця, місто, область, країна, поштовий індекс); на кроці 4 обирає спосіб оплати (банківський переказ, оплата при отриманні, кредитна картка, «купити зараз — заплатити пізніше», подарункова картка) і підтверджує замовлення. Підсумок замовлення містить суму товарів і вартість доставки. Вартість доставки визначається за BL-60: 120,00 грн; 0,00 грн, якщо сума після знижки не менша за 1500,00 грн. Рядки знижки за обсягом і за промокодом з’являються після інтеграції модуля (розділ 5) в інтерфейс. Застосування правила BL-60 до поточного інтерфейсу до інтеграції модуля та порядок урахування знижок потребують підтвердження замовником. Після підтвердження замовлення система показує повідомлення з номером рахунку-інвойсу.</x:v>
+        <x:v>Підсумок замовлення містить суму товарів і вартість доставки. Рядки знижки за обсягом і за промокодом з’являються після інтеграції модуля (розділ 5) в інтерфейс.</x:v>
       </x:c>
       <x:c r="F27" s="4" t="str">
         <x:v>Белінська Єлизавета (СМ)</x:v>
@@ -1182,7 +1182,7 @@
         <x:v>3. F-110; підстава 2.3</x:v>
       </x:c>
       <x:c r="I27" s="4" t="str">
-        <x:v>Потребує підтвердження замовником: Застосування BL-60 до поточного інтерфейсу і порядок урахування знижок.</x:v>
+        <x:v>Правка узгоджує склад підсумку з обмеженням §2.3; повний текст F-110 наведено у SRS 1.1.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="86" customHeight="1">
@@ -1225,7 +1225,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae4d02902d024c44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re83e84791e9b4dea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1494,10 +1494,10 @@
         <x:v>ID / місце</x:v>
       </x:c>
       <x:c r="C1" s="8" t="str">
-        <x:v>Критерій у джерелі</x:v>
+        <x:v>Критерій у поточній редакції</x:v>
       </x:c>
       <x:c r="D1" s="8" t="str">
-        <x:v>Опис і пункт чек-листа із джерела</x:v>
+        <x:v>Опис і пункт чек-листа</x:v>
       </x:c>
       <x:c r="E1" s="8" t="str">
         <x:v>Пропозиція із джерела</x:v>
@@ -1515,7 +1515,7 @@
         <x:v>№ дефекту</x:v>
       </x:c>
       <x:c r="J1" s="8" t="str">
-        <x:v>Рішення у джерелі / редакторська примітка</x:v>
+        <x:v>Поточна примітка / історія рішення</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="140" customHeight="1">
@@ -1582,7 +1582,7 @@
         <x:v>Прийнято: виправлення відрізняється від рядка 11 реєстру (склад підсумку, а не поріг доставки) — окремий дефект. → Реєстр № 26. Фінальний F-110 одночасно враховує №11 і №26; склад checkout і способи оплати збережено.</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="140" customHeight="1">
+    <x:row r="4" ht="142" customHeight="1">
       <x:c r="A4" s="4" t="str">
         <x:v>Д3</x:v>
       </x:c>
@@ -1590,10 +1590,10 @@
         <x:v>розд. 2.1</x:v>
       </x:c>
       <x:c r="C4" s="4" t="str">
-        <x:v>Повнота</x:v>
+        <x:v>Несуперечливість</x:v>
       </x:c>
       <x:c r="D4" s="4" t="str">
-        <x:v>Повнота (п. 2). Розд. 2.1: зареєстрованому покупцю доступні «промокоди», але в розд. 3 немає жодної F-вимоги на введення промокоду, а розд. 2.3 каже, що модуль, який їх перевіряє, не інтегрований в інтерфейс.</x:v>
+        <x:v>Несуперечливість (§4.4, п. 2). Розд. 2.1: зареєстрованому покупцю доступні «промокоди», але в розд. 3 немає жодної F-вимоги на введення промокоду, а розд. 2.3 каже, що модуль, який їх перевіряє, не інтегрований в інтерфейс.</x:v>
       </x:c>
       <x:c r="E4" s="4" t="str">
         <x:v>Розд. 2.1: прибрати «промокоди» з переліку функцій версії 1.0 і додати примітку «промокоди — після інтеграції модуля розд. 5».</x:v>
@@ -1611,7 +1611,9 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="J4" s="4" t="str">
-        <x:v>Прийнято, перекласифіковано з несуперечливості в «Повнота (п. 2)». → Реєстр № 27. Вихідне рішення наведено дослівно. Для фінального реєстру виконано редакторську класифікацію: «Несуперечливість, §4.4 п.2», за правилом §4.1. Число дефектів і автор не змінені.</x:v>
+        <x:v>Поточна редакторська класифікація: «Несуперечливість» (§4.4, п. 2).
+14.10.2026, Бойко Євгеній (ТА): після рев’ю від 13.10.2026 узгоджено класифікацію зі «Реєстром». За §4.1 головний критерій визначає виправлення: правка прибирає суперечність між переліком функцій §2.1 та обмеженням §2.3. Це редакторське узгодження.
+Історія командного рішення: Прийнято, перекласифіковано з несуперечливості в «Повнота (п. 2)». → Реєстр № 27.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="140" customHeight="1">
@@ -1884,7 +1886,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0153f4c7cc774f06"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra49a54c4520c4207"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>